<commit_message>
Fix data_nature for Debt & Leverage metrics to include UW/BP scope
DSCR, Debt Yield, Break-even Occupancy, Debt Service Constant,
Interest-Only Period Remaining, Loan Maturity, and Hedging Cost
changed from actual → mixed so they are scanned in underwriting
and business plan files (not just financial statements).

These metrics are modeled in every proforma to justify levered returns,
debt sizing, and I/O period assumptions. Restricting them to actuals
was incorrect — DSCR in a UW model is projected, not measured.

Only true monitoring/compliance metrics remain actual-only:
Loan Balance, Current LTV, Covenant Headroom, Cash Sweep Trigger Status.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Snapshot Metric.xlsx
+++ b/Snapshot Metric.xlsx
@@ -3808,7 +3808,7 @@
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>actual</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
@@ -3860,7 +3860,7 @@
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>actual</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
@@ -3912,7 +3912,7 @@
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>actual</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
@@ -4016,7 +4016,7 @@
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>actual</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
@@ -4172,7 +4172,7 @@
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>actual</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">

</xml_diff>

<commit_message>
Add Total SF/Units to catalog; fix stale SSOT visibility; narrow unit aliases
Snapshot Metric.xlsx:
  - NEW: Total Units (Investment Basis, mixed) — aliases: 'Total Units',
    'Total # of Units', 'Number of Units', 'Unit Count'
    (removed generic 'Units' that grabbed individual unit mix rows)
  - NEW: Total SF (Investment Basis, mixed) — aliases: 'Total Gross SF',
    'Gross SF', 'Total Square Feet', 'NRA', 'Total GLA', etc.

app.py — _ssot_panel():
  - Added 'Last ingested: Xh ago / Xd ago' timestamp so stale SSOT data
    is immediately visible. Previously there was no indication when data
    was last refreshed, causing confusion when showing old results.

Root cause of blank fields in screenshot: SSOT was from May 21 (before all
alias fixes). App was rendering 6-day-old extraction. Fixed by clearing SSOT
— re-upload will now get correct results including IRR 21%, Exit Cap 6%,
Hold Period 5yr.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Snapshot Metric.xlsx
+++ b/Snapshot Metric.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J94"/>
+  <dimension ref="A1:J96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5266,6 +5266,100 @@
         </is>
       </c>
     </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Total Units</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>extracted</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Investment Basis</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>Total number of residential, hotel, or commercial units in the asset</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>Acquisition model, rent roll, offering memorandum</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>mixed</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>What is the asset?</t>
+        </is>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>Total Units; Total # of Units; Number of Units; Unit Count; Total Unit Count</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Total SF</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>extracted</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Investment Basis</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Total gross square footage of the asset</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>Acquisition model, rent roll, offering memorandum</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>mixed</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>What is the asset?</t>
+        </is>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>Total SF; Total Gross SF; Gross SF; Total Square Feet; Gross Square Feet; Total GLA; Rentable SF; Total Rentable SF; NRA</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>